<commit_message>
Add newest game version (V27) index.html to repo root
Copy of 01_Ballistic_Bastion/Game_versions/2026-10-03_V27/index.html so the
game is on the first page of the GitHub repo. Logged in the file log (No 24).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RdrbvyFqjzTAEJXe6KXCn
</commit_message>
<xml_diff>
--- a/00_File_Log/JM_game_File_Log.xlsx
+++ b/00_File_Log/JM_game_File_Log.xlsx
@@ -296,7 +296,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FileLog" displayName="FileLog" ref="A1:L23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FileLog" displayName="FileLog" ref="A1:L24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A1:L23"/>
   <tableColumns count="12">
     <tableColumn id="1" name="No"/>
@@ -316,7 +316,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CurrentFiles" displayName="CurrentFiles" ref="A1:F9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CurrentFiles" displayName="CurrentFiles" ref="A1:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A1:F9"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Folder"/>
@@ -1731,14 +1731,14 @@
     </row>
     <row r="24" ht="15" customHeight="1" s="15">
       <c r="A24" s="17" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B24" s="18" t="n">
         <v>46298</v>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>04:03</t>
+          <t>04:06</t>
         </is>
       </c>
       <c r="D24" s="17" t="inlineStr">
@@ -1748,12 +1748,12 @@
       </c>
       <c r="E24" s="19" t="inlineStr">
         <is>
-          <t>JM_game</t>
+          <t>(GitHub root)</t>
         </is>
       </c>
       <c r="F24" s="19" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>index.html</t>
         </is>
       </c>
       <c r="G24" s="17" t="inlineStr">
@@ -1761,10 +1761,14 @@
           <t>Added</t>
         </is>
       </c>
-      <c r="H24" s="19" t="n"/>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>01_Ballistic_Bastion\Game_versions\2026-10-03_V27\index.html</t>
+        </is>
+      </c>
       <c r="I24" s="19" t="inlineStr">
         <is>
-          <t>Sync rules and repo conventions that every Claude session follows automatically</t>
+          <t>Newest game version (V27) copied to the repo root so it shows on the first page of GitHub</t>
         </is>
       </c>
       <c r="J24" s="17" t="inlineStr">
@@ -1772,10 +1776,14 @@
           <t>Claude session</t>
         </is>
       </c>
-      <c r="K24" s="17" t="n"/>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>V27</t>
+        </is>
+      </c>
       <c r="L24" s="19" t="inlineStr">
         <is>
-          <t>Requested by Merijn</t>
+          <t>Copy; the version folder stays the master. Replace this file when a newer version is made</t>
         </is>
       </c>
     </row>
@@ -8739,29 +8747,29 @@
     <row r="10" ht="15" customHeight="1" s="15">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>JM_game</t>
+          <t>(GitHub root)</t>
         </is>
       </c>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>CLAUDE.md</t>
+          <t>index.html</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Game (HTML)</t>
         </is>
       </c>
       <c r="D10" s="22">
-        <f>INDEX(Log!$B$2:$B$500,MATCH(23,Log!$A$2:$A$500,0))</f>
+        <f>INDEX(Log!$B$2:$B$500,MATCH(24,Log!$A$2:$A$500,0))</f>
         <v/>
       </c>
       <c r="E10" s="21" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
-          <t>Rules for Claude sessions (sync + conventions)</t>
+          <t>Copy of the newest game version (V27) for the GitHub front page</t>
         </is>
       </c>
     </row>

</xml_diff>